<commit_message>
docs(FCC): round-2 fixups — last two renames + README index to v1.1
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.1-2026-07-06.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.1-2026-07-06.xlsx
@@ -12941,7 +12941,7 @@
 |  Why this order?  &gt;          |
 |                              |
 |  With your order:            |
-|   Will it last   84% -&gt; 82%  |
+|   Will my money last   84% -&gt; 82%  |
 |   Lasts to age    92 -&gt; 90   |
 |   (estimates)                |
 |                              |
@@ -13058,7 +13058,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>'With your order: Will it last 84% → 82%, lasts to age 92 → 90 (estimates)' — suggested versus user order, side by side, before committing.</t>
+          <t>'With your order: Will my money last 84% → 82%, lasts to age 92 → 90 (estimates)' — suggested versus user order, side by side, before committing.</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(FCC): design chain APPROVED 2026-07-12 — build gate open
Founder finished the v1.1 pass with no comments. Cleared the 32 round-2
comments v1.1 had carried over in margin columns (already answered on
the review tab, which keeps the record). README statuses -> APPROVED.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.1-2026-07-06.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.1-2026-07-06.xlsx
@@ -5187,13 +5187,7 @@
 Screen reader order: greeting → hero as ONE sentence ('Your investments: 843,700 dollars, up 11,200 dollars this month, ahead of the market by half a percent, prices as of 4 pm') → each attention item as one sentence → will-it-last ('Likely, 84 percent, estimate. Opens Plan.'). Eye toggle announces 'Hide balances'/'Show balances' (pattern already in src/components/TopBar.tsx). All rows and buttons at least 44 points tall. Direction always word+arrow, never color alone. Hero number scales down via compact style (e.g. $842.3k) under large-type settings rather than truncating.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>"up $11,200 this month Triangle up" should be "Triangle (green color) up $11,200 this month"
-"Will it Last?" Is not clear if this is regarding retirement, and will it last till what age? 
-And info dots for investments, market, Net Worth.</t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -5302,11 +5296,7 @@
           <t>Must equal the Invest tab header total and the 'Investments' section of the Net worth tab, to the dollar</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Investment = stock + etfs + bonds + alternatives? It does not include cash or cash equivalents - Right?</t>
-        </is>
-      </c>
+      <c r="G7" s="3" t="n"/>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -5361,11 +5351,7 @@
           <t>Must equal the versus-market line on the Performance screen for the same period</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Benchmark in S&amp;P 500? If that add info dot</t>
-        </is>
-      </c>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -5739,11 +5725,7 @@
 Hero reads as one sentence: 'Safe to spend in July: 5,840 dollars, an estimate. 4,200 guaranteed from Social Security and pension, 1,640 safe to draw from savings. About 71,600 dollars this year.' Worth-a-look card announces 'Worth a look' first, then the fact — screen-reader tone matches visual calm. Larger default type for this lens (retiree eyes); all targets ≥44pt; breakdown uses tree lines PLUS the words Guaranteed/Safe draw, never indentation alone.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Re-evaluate the order of wordings - e.g. "Guaranteed $4200 Social Security + Pension" Norm is Social Security + Pension $4200 (Guaranteed) particularly with pay check but do your research. If it is suppose to be "Guaranteed Social Security $4200" That's perfect.</t>
-        </is>
-      </c>
+      <c r="G23" s="3" t="n"/>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -5825,11 +5807,7 @@
           <t>PIN: guaranteed + safe draw − big bills landing this month = the this-month figure to the dollar, on Home AND Cash flow (agreement test). The bills line appears on Home whenever it is non-zero — the card must visibly sum in every month.</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>What if safe draw is less the big bill. Where will that information be available?</t>
-        </is>
-      </c>
+      <c r="G26" s="3" t="n"/>
     </row>
     <row r="27" ht="46" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -6171,11 +6149,7 @@
           <t>The 'usual amount' shown here is the exact figure the rule used — stored on the flag at flag time, so the explanation never drifts from the decision</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>How are response formulated? Are we using LLM or theseare pre-crafted responses and app uses one the pre-crafted response just replacing $$$?</t>
-        </is>
-      </c>
+      <c r="G39" s="3" t="n"/>
     </row>
     <row r="40" ht="46" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -6345,11 +6319,7 @@
 Radio groups with full labels; the consequence sentence ('this sets up your Home and tab order') is read before the choices. Large targets; no time pressure.</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>What did yo u come for? - we should specifiy they can select multiple options as retired person can still ne interested in growing her investments or see everything in one place. (2) When person first download Finwise - should we tell user what Finwise can do?</t>
-        </is>
-      </c>
+      <c r="G46" s="3" t="n"/>
     </row>
     <row r="47" ht="46" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
@@ -6431,11 +6401,7 @@
           <t>Skipping never produces different numbers — only default ordering.</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>If user select "just explore" - what's the next few screens they will see?</t>
-        </is>
-      </c>
+      <c r="G49" s="3" t="n"/>
     </row>
     <row r="50" ht="46" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -6529,11 +6495,7 @@
 Both doors are full-width ≥48pt buttons announced with their sub-lines ('Connect your first account, takes about 2 minutes, read-only'). Illustration marked decorative (skipped by screen readers). Preview list is a proper list for rotor navigation.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>"your whole picture in one place" - your whole picture not clear - may be your entire finance picture or some thing? Same for "the few things need you, in dollars" - not sure what you mean by in dollars?</t>
-        </is>
-      </c>
+      <c r="G53" s="3" t="n"/>
     </row>
     <row r="54" ht="46" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
@@ -6764,11 +6726,7 @@
 Masked values announce as 'hidden' (not 'bullet bullet bullet'). Eye announces 'Show balances' when hidden — labels already exist in src/components/TopBar.tsx. The banner is polite-priority for screen readers (announced once, not repeated per element).</t>
         </is>
       </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>This does not have refresh date and time.</t>
-        </is>
-      </c>
+      <c r="G62" s="3" t="n"/>
     </row>
     <row r="63" ht="46" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
@@ -6944,11 +6902,7 @@
 Banner is announced once on arrival ('Information: Chase hasn't updated since June 27'), not on every scroll. Stamps are part of each number's spoken sentence ('…as of June 27'). Info icon always paired with words. Fix button ≥44pt.</t>
         </is>
       </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>in mock up 1 - date and time was after "your investments" and before " Net Worth", here it is after "net worth". Which is the right place?</t>
-        </is>
-      </c>
+      <c r="G69" s="3" t="n"/>
     </row>
     <row r="70" ht="46" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
@@ -7145,11 +7099,7 @@
 Read as one story: fact, where, comparison. Rates always paired with the word estimate.</t>
         </is>
       </c>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>From where comparative data coming? Do we have analytical engine built to analyze all imported data and come up with these insights?</t>
-        </is>
-      </c>
+      <c r="G77" s="3" t="n"/>
     </row>
     <row r="78" ht="40" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
@@ -7361,6 +7311,7 @@
       <c r="D86" s="4" t="n"/>
       <c r="E86" s="4" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88" ht="42" customHeight="1">
       <c r="A88" s="5" t="inlineStr">
         <is>
@@ -7601,11 +7552,7 @@
 Every row is a button whose spoken label includes name, amount, source and last-updated ('Fidelity Brokerage, $521,300, connected, updated today 6:04 am'). Own/owe conveyed by section words and minus signs, never color alone; paused connections say 'paused' in text. All targets at least 44 points; text scales with system size; the trend line carries a one-sentence spoken summary.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double check in strategy and design document - did we say that people think in terms of non-retirement and retirement accounts? If yes, do we want to list retirement account as Retirement account (401K/IRA/etc.). We should have info dots for all asset classes. </t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -7633,11 +7580,7 @@
           <t>The exact number shown on Home and everywhere else — every surface calls buildNetWorth(totalAssets, totalDebtBalance); pinned by the cross-screen agreement test (src/domain/assets/agreement.test.ts).</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Plain line - means line graph?</t>
-        </is>
-      </c>
+      <c r="G4" s="3" t="n"/>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -7773,11 +7716,7 @@
           <t>The stamp describes freshness only; the amount itself is always the stored balance that totalAssets sums — stale never means different.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>what does screen look like for manual update?</t>
-        </is>
-      </c>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -7832,11 +7771,7 @@
           <t>All three paths write accounts through the same store.addAsset / store.updateAsset actions (src/store/useStore.ts), so a linked, imported, or hand-typed account is the same kind of row everywhere.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review the Add account screen to make sure it we have separate screen or dynamic screen adjusting by asset class ensuring we are collecting right and required information. </t>
-        </is>
-      </c>
+      <c r="G11" s="3" t="n"/>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -7891,11 +7826,7 @@
           <t>cashTotal is the same canonical cash number as the Cash row above it; plannedMonthlySpend is the same budget figure the Plan tab uses.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Cash = cash + cash equivalent?</t>
-        </is>
-      </c>
+      <c r="G13" s="3" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -7923,11 +7854,7 @@
           <t>PIN: identical projection to Plan's will-it-last detail band and Invest's forward what-if baseline — one engine, one assumptions source; TODAY's balances never move on adoption (futures only).</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>is the display graph, table, or just numbers?</t>
-        </is>
-      </c>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15" ht="64" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -8057,11 +7984,7 @@
 Consent card is real text (not an image), scales with system size, and is read in full by the screen reader before the Continue button. Buttons are labeled with outcomes ('Continue to Plaid to sign in to Fidelity, read-only'). Progress states are announced. Color never carries meaning alone.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>import from a file - do we need specific format if yes, we should specify. May be have a info dot to explain file type and must have columns?</t>
-        </is>
-      </c>
+      <c r="G19" s="3" t="n"/>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -8317,11 +8240,7 @@
           <t>Linked accounts enter the same accounts array every total reads — totalAssets, assetAllocation and buildNetWorth pick them up with zero new math.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>do we capture only balance or all individual portfolio holding e.g. AMZN 100 stocks ….</t>
-        </is>
-      </c>
+      <c r="G29" s="3" t="n"/>
     </row>
     <row r="30" ht="46" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -8730,11 +8649,7 @@
 Action buttons say their outcome ('Record a deposit into Chase Checking'). History rows read as full sentences with signed amounts spoken as 'minus five thousand two hundred dollars'. The stale-value nudge is a labeled alert, and the paused state is announced in words. All amounts respect hidden-balances in spoken output too.</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>When dividend is captured is it automatically added to income or cash? Similarly, is there a way captical gain is captured and displayed somewhere?</t>
-        </is>
-      </c>
+      <c r="G45" s="3" t="n"/>
     </row>
     <row r="46" ht="46" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
@@ -8965,11 +8880,7 @@
 Every field labeled; the maturity picker announces the chosen date (existing accessibility label kept). The 12-month cash-vs-bond rule is stated in visible text under the date, not hidden in a tooltip. Sale confirmations read the full sentence including both values. Nudges are announced alerts.</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Is it imported directly using Plaid? Also, Does it capture interest payment for bonds? </t>
-        </is>
-      </c>
+      <c r="G54" s="3" t="n"/>
     </row>
     <row r="55" ht="46" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -9227,11 +9138,7 @@
 Chips are toggle buttons with selected state announced. Hints are visible text, not tooltips. Sale/close confirmations read as full sentences with both values. The staleness nudge is an announced alert paired with the clock icon and words.</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Is this manual, imported or connected and captured via Plaid? </t>
-        </is>
-      </c>
+      <c r="G64" s="3" t="n"/>
     </row>
     <row r="65" ht="46" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
@@ -9361,6 +9268,7 @@
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="n"/>
     </row>
+    <row r="70"/>
     <row r="71" ht="42" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
@@ -9669,11 +9577,7 @@
 Gains/losses always carry the word 'up'/'down' plus an arrow icon — never red/green alone (colorblind-safe). Every row is one tap target 44pt+ with a spoken label like 'NVIDIA, $261,900, up 41 percent this year'. Period selector is a radio group announced as 'showing 1 year'. The trend chart has a text summary ('you +12.9%, market +10.1%') so screen readers don't need the picture.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Total return captures both realized and unrealized gains? Is there any place we display realized P/L, unrealized P/L, total dividend, and total interest separately?</t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -9917,11 +9821,7 @@
           <t>The group subtotals and $843,700 total are the same balances Net Worth shows — recomputeBalances (src/store/useStore.ts:13) is the single writer of balance; pinned by the assets agreement test (src/domain/assets/agreement.test.ts).</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Is this expandable / collapasable as many people can have 20-30 or more holdings?</t>
-        </is>
-      </c>
+      <c r="G12" s="3" t="n"/>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -9976,11 +9876,7 @@
           <t>n/a (navigation)</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>What's the objective of "what if" - evaluate what if I had bought Nvidia instead of Amazon 6 months ago or something different?</t>
-        </is>
-      </c>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -10008,11 +9904,7 @@
           <t>PIN: equals the Plan hub's committed saving and the Cash flow planned line — one shared source (F11).</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>How do we evaluate if something is saved towards retirement or some other goals? In other words is NW = Retire or Retire = Assets - Primary home - primary car?</t>
-        </is>
-      </c>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16" ht="64" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -10164,11 +10056,7 @@
 Header spoken as one sentence: 'NVIDIA, worth $261,900, up $76,200, 41 percent since purchase'. 'Ahead by 30.9 points' uses the word 'ahead', not color. Estimate labels are real text, not just styling, so screen readers hear them.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>stocks with dividends - will it also show dividends received?</t>
-        </is>
-      </c>
+      <c r="G21" s="3" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -11386,11 +11274,7 @@
 Type chips are a radio group. Guardrail messages are polite live-region announcements ('This buy costs more than the cash available'). History rows read as full sentences including the date.</t>
         </is>
       </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>If an account is connected but someone adds transaction manually - is that allowed and how will the reconciliation between captured info from Plaid versus manual entry happen?</t>
-        </is>
-      </c>
+      <c r="G69" s="3" t="n"/>
     </row>
     <row r="70" ht="46" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
@@ -12206,11 +12090,7 @@
 Surplus announced with direction words ('one thousand seven hundred forty dollars ahead'). Projection card is announced with its estimate disclaimer first. Bars carry full per-month spoken values.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>What's the flow to add actual day to day expenses such grocery, gas, etc? Also, what's the flow to capture or add income?</t>
-        </is>
-      </c>
+      <c r="G16" s="3" t="n"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -13588,11 +13468,7 @@
 Chance always pairs the percent with a word (Likely / Uncertain / Unlikely) so color never carries meaning alone. Band chart has a text alternative ('in the worst 1-in-10 futures, 71%'). All rows are one full-width tap target, minimum 44 points tall. Screen-reader order: headline, decisions, scenarios, revert, sharpen.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>"will it last" should it specify that this is about retirement? Right now it is not clear - what will last, and till when?</t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -13774,6 +13650,7 @@
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -13899,11 +13776,7 @@
           <t>PIN: the '67' row always equals the statement amount exactly (the factor at full claiming age is 1.0) -- a unit test pins this so the table can never drift from the user's own input.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>How is the amount calculated by age? Is this a formula used by social security administration?</t>
-        </is>
-      </c>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="3" t="inlineStr">

</xml_diff>